<commit_message>
Redact personal contact details from aerial photos spreadsheet
</commit_message>
<xml_diff>
--- a/08_Operational_History_and_Traffic/CEMEX aerial photos EXCEL.xlsx
+++ b/08_Operational_History_and_Traffic/CEMEX aerial photos EXCEL.xlsx
@@ -1,216 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="36">
-  <si>
-    <t>Table 1</t>
-  </si>
-  <si>
-    <t>AERIAL PHOTOS</t>
-  </si>
-  <si>
-    <t>SOURCE</t>
-  </si>
-  <si>
-    <t>WEBSITE</t>
-  </si>
-  <si>
-    <t>DATES</t>
-  </si>
-  <si>
-    <t>FORMAT</t>
-  </si>
-  <si>
-    <t>COMMENTS</t>
-  </si>
-  <si>
-    <t>SEARCH TIP</t>
-  </si>
-  <si>
-    <t>Boulder County Assessor’s Office Property Search</t>
-  </si>
-  <si>
-    <t>maps.boco.solutions</t>
-  </si>
-  <si>
-    <t>2020, 2018, 2016, 2014, 2013, 2010, 2008, older?</t>
-  </si>
-  <si>
-    <t>onscreen</t>
-  </si>
-  <si>
-    <t>Easy to browse back and forth across images, but I see no mapping functions or ways to download images.</t>
-  </si>
-  <si>
-    <t>Search on Acct # P0204735 or address 5134 Ute Hwy, Lyons, CO</t>
-  </si>
-  <si>
-    <t>Google Earth</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>earth.google.com</t>
-    </r>
-  </si>
-  <si>
-    <t>many dates between 2023 and 2005 (some w clouds or snow);  2003, 2002, 1999, 1985</t>
-  </si>
-  <si>
-    <t>Excellent zoom onscreen. Very good resolution on many images. Pretty easy to use, but I don’t know how to export images for comparative mapping. I’m hoping to figure out how to use the Timelapse function, and possibly zoom in for max detail.  Not sure yet if older imagery is available.</t>
-  </si>
-  <si>
-    <t>Search on CEMEX, Lyons, CO</t>
-  </si>
-  <si>
-    <t>NETRonline Historic Aerials</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>www.historic</t>
-    </r>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>aerials.com</t>
-    </r>
-  </si>
-  <si>
-    <t>2021, 2019, 2017, 2015, 2013, 2011, 2009, 2004, 1999, 1983, 1978, 1971, and earlier</t>
-  </si>
-  <si>
-    <t>order prints or digital images</t>
-  </si>
-  <si>
-    <t>Orthorectified images with variable resolution. No stereo coverage. Excellent detail on many images. Easy to order prints or digital files for use in mapping. I have contacted Jeff Teasley, Director of Historic Aerials, 480-967-6752 X006 in Tempe, AZ, for more info and I plan to call him on Monday.</t>
-  </si>
-  <si>
-    <t>Search on address 5134 Ute Hwy, Lyons, CO</t>
-  </si>
-  <si>
-    <t>USGS Earth Explorer</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>earthexplorer.usgs.gov</t>
-    </r>
-  </si>
-  <si>
-    <t>MANY!!</t>
-  </si>
-  <si>
-    <t>Order digital or prints from many available programs: National Aerial Photography Program (NAPP), National High Altitude Photography (NHAP), Digital Orthophoto Quadrangles (DOQ), and many other data set choices, including Landsat (satellite) imagery</t>
-  </si>
-  <si>
-    <t>LOTS of coverages but I have yet to find good resolution for comparing features of the factory, even on lower altitude photos. Considerable research will be needed to find any gems in these data sets. Probably stereo coverage in some formats. Satellite imagery may be our best options, if resolution is adequate and cloud cover minimal. Cust service is 605-594-6151 in Sioux Falls, SD. I can call them Monday to see if we can get a better idea what might be useful here.</t>
-  </si>
-  <si>
-    <t>Search on circle: center lat 40.2021 long -105.2367, radius 800 meters</t>
-  </si>
-  <si>
-    <t>ALSO…</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t xml:space="preserve">updated 1/3/2025, by Kit Fuller, </t>
-    </r>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>fullerhkit@yahoo.com</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>, 720-440-3276</t>
-    </r>
-  </si>
-  <si>
-    <t>OTHER NOTES</t>
-  </si>
-  <si>
-    <t>In addition to this information, Brianne at the Carnegie Library in Boulder is contacting a few people to see if there are other options available.</t>
-  </si>
-  <si>
-    <t>I have also looked online at the CU Library, which may have aerial photos available for viewing, but they are closed until Monday.</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
+      <name val="Helvetica Neue"/>
+      <color indexed="8"/>
       <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
       <b val="1"/>
+      <color indexed="8"/>
       <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
+      <color indexed="8"/>
+      <sz val="10"/>
       <u val="single"/>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
     </font>
   </fonts>
   <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -343,62 +174,62 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+  <cellXfs count="16">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="ff000000"/>
@@ -1441,238 +1272,313 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:F16"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="1" width="16.3516" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.1328" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7266" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5859" style="1" customWidth="1"/>
-    <col min="5" max="5" width="25.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.3516" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="16.3516" style="1" customWidth="1"/>
+    <col width="16.3516" customWidth="1" style="1" min="1" max="1"/>
+    <col width="16.1328" customWidth="1" style="1" min="2" max="2"/>
+    <col width="10.7266" customWidth="1" style="1" min="3" max="3"/>
+    <col width="14.5859" customWidth="1" style="1" min="4" max="4"/>
+    <col width="25.5" customWidth="1" style="1" min="5" max="5"/>
+    <col width="16.3516" customWidth="1" style="1" min="6" max="6"/>
+    <col width="16.3516" customWidth="1" style="1" min="7" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.65" customHeight="1">
-      <c r="A1" t="s" s="2">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+    <row r="1" ht="27.65" customHeight="1" s="15">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
     </row>
-    <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" t="s" s="3">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+    <row r="2" ht="20.25" customHeight="1" s="15">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>AERIAL PHOTOS</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
     </row>
-    <row r="3" ht="20.25" customHeight="1">
-      <c r="A3" t="s" s="5">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s" s="6">
-        <v>3</v>
-      </c>
-      <c r="C3" t="s" s="7">
-        <v>4</v>
-      </c>
-      <c r="D3" t="s" s="7">
-        <v>5</v>
-      </c>
-      <c r="E3" t="s" s="7">
-        <v>6</v>
-      </c>
-      <c r="F3" t="s" s="7">
-        <v>7</v>
+    <row r="3" ht="20.25" customHeight="1" s="15">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>WEBSITE</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>DATES</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>FORMAT</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>COMMENTS</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>SEARCH TIP</t>
+        </is>
       </c>
     </row>
-    <row r="4" ht="56.05" customHeight="1">
-      <c r="A4" t="s" s="8">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s" s="10">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s" s="10">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s" s="10">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s" s="10">
-        <v>13</v>
+    <row r="4" ht="56.05" customHeight="1" s="15">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Boulder County Assessor’s Office Property Search</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>maps.boco.solutions</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>2020, 2018, 2016, 2014, 2013, 2010, 2008, older?</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>onscreen</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Easy to browse back and forth across images, but I see no mapping functions or ways to download images.</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Search on Acct # P0204735 or address 5134 Ute Hwy, Lyons, CO</t>
+        </is>
       </c>
     </row>
-    <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" s="11"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
+    <row r="5" ht="20.05" customHeight="1" s="15">
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="12" t="n"/>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="13" t="n"/>
     </row>
-    <row r="6" ht="128.05" customHeight="1">
-      <c r="A6" t="s" s="8">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s" s="9">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s" s="10">
-        <v>16</v>
-      </c>
-      <c r="D6" t="s" s="10">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s" s="10">
-        <v>17</v>
-      </c>
-      <c r="F6" t="s" s="10">
-        <v>18</v>
+    <row r="6" ht="128.05" customHeight="1" s="15">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Google Earth</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>earth.google.com</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>many dates between 2023 and 2005 (some w clouds or snow);  2003, 2002, 1999, 1985</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>onscreen</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Excellent zoom onscreen. Very good resolution on many images. Pretty easy to use, but I don’t know how to export images for comparative mapping. I’m hoping to figure out how to use the Timelapse function, and possibly zoom in for max detail.  Not sure yet if older imagery is available.</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Search on CEMEX, Lyons, CO</t>
+        </is>
       </c>
     </row>
-    <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" s="11"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
+    <row r="7" ht="20.05" customHeight="1" s="15">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="12" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="13" t="n"/>
     </row>
-    <row r="8" ht="128.05" customHeight="1">
-      <c r="A8" t="s" s="8">
-        <v>19</v>
-      </c>
-      <c r="B8" t="s" s="9">
-        <v>20</v>
-      </c>
-      <c r="C8" t="s" s="10">
-        <v>21</v>
-      </c>
-      <c r="D8" t="s" s="10">
-        <v>22</v>
-      </c>
-      <c r="E8" t="s" s="10">
-        <v>23</v>
-      </c>
-      <c r="F8" t="s" s="10">
-        <v>24</v>
+    <row r="8" ht="128.05" customHeight="1" s="15">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>NETRonline Historic Aerials</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>www.historicaerials.com</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>2021, 2019, 2017, 2015, 2013, 2011, 2009, 2004, 1999, 1983, 1978, 1971, and earlier</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>order prints or digital images</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Orthorectified images with variable resolution. No stereo coverage. Excellent detail on many images. Easy to order prints or digital files for use in mapping. I have contacted [redacted], Director of Historic Aerials, [redacted] in Tempe, AZ, for more info and I plan to call him on Monday.</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Search on address 5134 Ute Hwy, Lyons, CO</t>
+        </is>
       </c>
     </row>
-    <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
+    <row r="9" ht="20.05" customHeight="1" s="15">
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
     </row>
-    <row r="10" ht="224.05" customHeight="1">
-      <c r="A10" t="s" s="8">
-        <v>25</v>
-      </c>
-      <c r="B10" t="s" s="9">
-        <v>26</v>
-      </c>
-      <c r="C10" t="s" s="10">
-        <v>27</v>
-      </c>
-      <c r="D10" t="s" s="10">
-        <v>28</v>
-      </c>
-      <c r="E10" t="s" s="10">
-        <v>29</v>
-      </c>
-      <c r="F10" t="s" s="10">
-        <v>30</v>
+    <row r="10" ht="224.05" customHeight="1" s="15">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>USGS Earth Explorer</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>earthexplorer.usgs.gov</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>MANY!!</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Order digital or prints from many available programs: National Aerial Photography Program (NAPP), National High Altitude Photography (NHAP), Digital Orthophoto Quadrangles (DOQ), and many other data set choices, including Landsat (satellite) imagery</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>LOTS of coverages but I have yet to find good resolution for comparing features of the factory, even on lower altitude photos. Considerable research will be needed to find any gems in these data sets. Probably stereo coverage in some formats. Satellite imagery may be our best options, if resolution is adequate and cloud cover minimal. Cust service is [redacted] in Sioux Falls, SD. I can call them Monday to see if we can get a better idea what might be useful here.</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Search on circle: center lat 40.2021 long -105.2367, radius 800 meters</t>
+        </is>
       </c>
     </row>
-    <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
+    <row r="11" ht="20.05" customHeight="1" s="15">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
     </row>
-    <row r="12" ht="68.05" customHeight="1">
-      <c r="A12" t="s" s="8">
-        <v>31</v>
-      </c>
-      <c r="B12" t="s" s="9">
-        <v>32</v>
-      </c>
-      <c r="C12" s="13"/>
-      <c r="D12" t="s" s="14">
-        <v>33</v>
-      </c>
-      <c r="E12" t="s" s="10">
-        <v>34</v>
-      </c>
-      <c r="F12" s="13"/>
+    <row r="12" ht="68.05" customHeight="1" s="15">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>ALSO…</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>updated 1/3/2025, by [redacted], [redacted], [redacted]</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>OTHER NOTES</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>In addition to this information, [redacted] at the Carnegie Library in Boulder is contacting a few people to see if there are other options available.</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="n"/>
     </row>
-    <row r="13" ht="68.05" customHeight="1">
-      <c r="A13" s="11"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" t="s" s="10">
-        <v>35</v>
-      </c>
-      <c r="F13" s="13"/>
+    <row r="13" ht="68.05" customHeight="1" s="15">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>I have also looked online at the CU Library, which may have aerial photos available for viewing, but they are closed until Monday.</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="n"/>
     </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="11"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
+    <row r="14" ht="20.05" customHeight="1" s="15">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
     </row>
-    <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" s="11"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
+    <row r="15" ht="20.05" customHeight="1" s="15">
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13" t="n"/>
     </row>
-    <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" s="11"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
+    <row r="16" ht="20.05" customHeight="1" s="15">
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" location="" tooltip="" display="earth.google.com"/>
-    <hyperlink ref="B8" r:id="rId2" location="" tooltip="" display="aerials.com"/>
-    <hyperlink ref="B10" r:id="rId3" location="" tooltip="" display="earthexplorer.usgs.gov"/>
-    <hyperlink ref="B12" r:id="rId4" location="" tooltip="" display="fullerhkit@yahoo.com"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" location="" tooltip="" display="earth.google.com" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" location="" tooltip="" display="aerials.com" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" location="" tooltip="" display="earthexplorer.usgs.gov" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" location="" tooltip="" display="fullerhkit@yahoo.com" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
   <headerFooter>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12 &amp;K000000&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>